<commit_message>
fix(ghost-kitchen-checklists-en): ronda 1 de la revisión adversarial — 4 MAYOR + 18 menor aplicados
Aceite según TPM con boil-out, las tres opciones de 3-402.11 completas, verano = temporada baja del delivery,
impresora/cartas/86 antes de encender las marcas, utensilios cada 4 h, sonda diaria, trampa de grasa.
Landing alineada. 6 hermanos idénticos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/ghost-kitchen-checklist-templates/01-ghost-kitchen-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/ghost-kitchen-checklist-templates/01-ghost-kitchen-opening-closing-checklists.xlsx
@@ -1186,9 +1186,9 @@
       <c r="A18" s="25" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="26" t="inlineStr">
-        <is>
-          <t>Set up mise en place for all brands/concepts</t>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>Set up mise en place for all brands/concepts, on surfaces already cleaned and sanitized (task #30)</t>
         </is>
       </c>
       <c r="C18" s="27" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="E31" s="27" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="F31" s="28" t="n"/>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="E32" s="27" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="F32" s="28" t="n"/>
@@ -1563,9 +1563,9 @@
       <c r="A33" s="29" t="n">
         <v>24</v>
       </c>
-      <c r="B33" s="34" t="inlineStr">
-        <is>
-          <t>Turn on all brands in DoorDash, Uber Eats and Grubhub</t>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>Check the ticket printer works</t>
         </is>
       </c>
       <c r="C33" s="27" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="E33" s="27" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>10:15 AM</t>
         </is>
       </c>
       <c r="F33" s="28" t="n"/>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="E34" s="27" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>10:15 AM</t>
         </is>
       </c>
       <c r="F34" s="28" t="n"/>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="E35" s="27" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>10:15 AM</t>
         </is>
       </c>
       <c r="F35" s="28" t="n"/>
@@ -1644,9 +1644,9 @@
       <c r="A36" s="29" t="n">
         <v>27</v>
       </c>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>Check the ticket printer works</t>
+      <c r="B36" s="34" t="inlineStr">
+        <is>
+          <t>86 anything out of stock: pause that dish or brand in each app</t>
         </is>
       </c>
       <c r="C36" s="27" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="B37" s="33" t="inlineStr">
         <is>
-          <t>86 anything out of stock: pause that dish or brand in each app</t>
+          <t>Turn on all brands in DoorDash, Uber Eats and Grubhub — last, once the tablets, printer, menus and 86s are checked</t>
         </is>
       </c>
       <c r="C37" s="27" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>Date-mark all prepped food (ready-to-eat keeps 7 days at 41 °F; prep day = day 1)</t>
+          <t>Date-mark all prepped food: prep day = day 1, 7 days max at 41 °F (FDA 3-501.17), or less where the "Weekly FIFO Check" tab in 05 sets a shorter limit</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>Filter or change the fryer oil if due, per the fryer manufacturer's instructions (many have built-in filtration designed for hot oil; others need it cooled), with heat-resistant gloves, apron and goggles; used oil goes to the used cooking oil recycler's container</t>
+          <t>Filter the fryer oil per the fryer manufacturer (many have built-in filtration designed for hot oil; others need it cooled) and change it when the TPM tester says, with heat-resistant gloves, apron and goggles; used oil goes to the used cooking oil recycler's container</t>
         </is>
       </c>
       <c r="C13" s="27" t="inlineStr">

</xml_diff>